<commit_message>
Switch the calculator to September and pay every hour worked
The Dienstplan sheet now carries the September roster read off the
Supershift screenshot: 10 TD and 5 ND, 15 shifts of 12 h = 180 h, of
which 36 h are night-only and 28 h Sunday (14 night hours fall on a
Sunday and are paid at the higher Sunday rate instead).

Sets the pauschal overtime allowance to 0 so the model mirrors what
the employer actually pays. The August payslip settled all 216 hours
rather than deducting the 8 hours § 2 Abs. 3 would allow, and the
calculator was understating gross by that difference.

The August reconciliation no longer reads its hours from Dienstplan,
which now holds a different month; those three figures are written
out as constants so the comparison keeps standing on its own.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NKeNmKEfCtXiZJGvjE51Zk
</commit_message>
<xml_diff>
--- a/Gehaltsrechner_Karimov.xlsx
+++ b/Gehaltsrechner_Karimov.xlsx
@@ -816,7 +816,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>График месяца: ND / TD / FREI, статус (Arbeit / Urlaub / Krank), «x» = Eingesprungen. Август 2026 заполнен по факту: 18 смен = 216 ч.</t>
+          <t>График месяца: ND / TD / FREI, статус (Arbeit / Urlaub / Krank), «x» = Eingesprungen. Сейчас заполнен СЕНТЯБРЬ 2026: 10 TD + 5 ND = 15 смен = 180 ч.</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="26" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Сверка с расчёткой</t>
@@ -912,7 +912,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Реальные Lohnabrechnung 07/2026 и 08/2026, разобранные построчно, и проверка каждой суммы.</t>
+          <t>Реальные Lohnabrechnung 07/2026 и 08/2026, разобранные построчно, и проверка каждой суммы. Август зафиксирован числами и не меняется при смене месяца.</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
     <row r="21" ht="19" customHeight="1">
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>АВГУСТ — СХОДЯТСЯ ЛИ ЧАСЫ С ГРАФИКОМ</t>
+          <t>АВГУСТ — СХОДЯТСЯ ЛИ ЧАСЫ (числа зафиксированы, лист Dienstplan уже за сентябрь)</t>
         </is>
       </c>
     </row>
@@ -2047,15 +2047,14 @@
     <row r="23">
       <c r="B23" s="64" t="inlineStr">
         <is>
-          <t>Смен по графику (лист Dienstplan)</t>
+          <t>Отработано по графику</t>
         </is>
       </c>
       <c r="C23" s="73" t="n"/>
       <c r="D23" s="73" t="n"/>
       <c r="E23" s="73" t="n"/>
-      <c r="F23" s="75">
-        <f>Dienstplan!$L$36</f>
-        <v/>
+      <c r="F23" s="75" t="n">
+        <v>216</v>
       </c>
       <c r="G23" s="73" t="n"/>
       <c r="H23" s="8" t="inlineStr">
@@ -2112,9 +2111,8 @@
       <c r="C26" s="73" t="n"/>
       <c r="D26" s="73" t="n"/>
       <c r="E26" s="73" t="n"/>
-      <c r="F26" s="75">
-        <f>Dienstplan!$AM$36</f>
-        <v/>
+      <c r="F26" s="75" t="n">
+        <v>132</v>
       </c>
       <c r="G26" s="73" t="n"/>
       <c r="H26" s="8" t="inlineStr">
@@ -2132,9 +2130,8 @@
       <c r="C27" s="73" t="n"/>
       <c r="D27" s="73" t="n"/>
       <c r="E27" s="73" t="n"/>
-      <c r="F27" s="75">
-        <f>Dienstplan!$M$36-Dienstplan!$AM$36</f>
-        <v/>
+      <c r="F27" s="75" t="n">
+        <v>28</v>
       </c>
       <c r="G27" s="73" t="n"/>
       <c r="H27" s="8" t="inlineStr">
@@ -2167,9 +2164,8 @@
       <c r="C29" s="73" t="n"/>
       <c r="D29" s="73" t="n"/>
       <c r="E29" s="73" t="n"/>
-      <c r="F29" s="75">
-        <f>Dienstplan!$N$36</f>
-        <v/>
+      <c r="F29" s="75" t="n">
+        <v>44</v>
       </c>
       <c r="G29" s="73" t="n"/>
       <c r="H29" s="8" t="inlineStr"/>
@@ -2206,7 +2202,7 @@
     <row r="34" ht="52" customHeight="1">
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Работодатель заплатил ЩЕДРЕЕ, чем написано в договоре: § 2 Abs. 3 разрешает не платить первые 8 ч переработки в месяц, но в расчётке оплачены все 216 ч (168 + 48), а не 208. Это +216,00 € брутто в твою пользу. Лист «Расчёт» считает строго по договору, поэтому там брутто 7.101 €, а в расчётке 7.317 €. Если хочешь, чтобы файл повторял расчётку точь-в-точь, поставь в «Настройках» «Переработка включена в оклад» = 0.</t>
+          <t>Работодатель заплатил ЩЕДРЕЕ, чем написано в договоре: § 2 Abs. 3 разрешает не платить первые 8 ч переработки в месяц, но в расчётке оплачены все 216 ч (168 + 48), а не 208. Это +216,00 € брутто в твою пользу. Поэтому в «Настройках» «Переработка включена в оклад» стоит 0 — так файл повторяет расчётку. Поставь 8, если захочешь увидеть, сколько работодатель обязан минимум по договору.</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2757,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
     </row>
@@ -2904,11 +2900,11 @@
         </is>
       </c>
       <c r="D14" s="14" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>§ 2 Abs. 3 — до 8 ч/мес уже в окладе</t>
+          <t>§ 2 Abs. 3 договора разрешает не платить первые 8 ч/мес. Но в расчётке 08/2026 оплачены ВСЕ 216 ч — поэтому здесь 0. Поставь 8, если хочешь увидеть минимум по договору</t>
         </is>
       </c>
     </row>
@@ -4757,10 +4753,14 @@
       </c>
       <c r="D5" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E5" s="30" t="inlineStr"/>
+          <t>TD</t>
+        </is>
+      </c>
+      <c r="E5" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
       <c r="F5" s="30" t="inlineStr"/>
       <c r="G5" s="30" t="inlineStr"/>
       <c r="H5" s="31">
@@ -4908,7 +4908,7 @@
       </c>
       <c r="D6" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>TD</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
@@ -5066,14 +5066,10 @@
       </c>
       <c r="D7" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E7" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E7" s="30" t="inlineStr"/>
       <c r="F7" s="30" t="inlineStr"/>
       <c r="G7" s="30" t="inlineStr"/>
       <c r="H7" s="31">
@@ -5540,10 +5536,14 @@
       </c>
       <c r="D10" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E10" s="30" t="inlineStr"/>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
       <c r="F10" s="30" t="inlineStr"/>
       <c r="G10" s="30" t="inlineStr"/>
       <c r="H10" s="31">
@@ -6002,7 +6002,7 @@
       </c>
       <c r="D13" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>TD</t>
         </is>
       </c>
       <c r="E13" s="30" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="D14" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>TD</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -6318,7 +6318,7 @@
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>TD</t>
         </is>
       </c>
       <c r="E15" s="30" t="inlineStr">
@@ -6476,7 +6476,7 @@
       </c>
       <c r="D16" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>TD</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -6634,10 +6634,14 @@
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E17" s="30" t="inlineStr"/>
+          <t>TD</t>
+        </is>
+      </c>
+      <c r="E17" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
       <c r="F17" s="30" t="inlineStr"/>
       <c r="G17" s="30" t="inlineStr"/>
       <c r="H17" s="31">
@@ -6788,10 +6792,14 @@
       </c>
       <c r="D18" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E18" s="30" t="inlineStr"/>
+          <t>TD</t>
+        </is>
+      </c>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
       <c r="F18" s="30" t="inlineStr"/>
       <c r="G18" s="30" t="inlineStr"/>
       <c r="H18" s="31">
@@ -6942,14 +6950,10 @@
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E19" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E19" s="30" t="inlineStr"/>
       <c r="F19" s="30" t="inlineStr"/>
       <c r="G19" s="30" t="inlineStr"/>
       <c r="H19" s="31">
@@ -7100,14 +7104,10 @@
       </c>
       <c r="D20" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E20" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="inlineStr"/>
       <c r="F20" s="30" t="inlineStr"/>
       <c r="G20" s="30" t="inlineStr"/>
       <c r="H20" s="31">
@@ -8028,14 +8028,10 @@
       </c>
       <c r="D26" s="30" t="inlineStr">
         <is>
-          <t>TD</t>
-        </is>
-      </c>
-      <c r="E26" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E26" s="30" t="inlineStr"/>
       <c r="F26" s="30" t="inlineStr"/>
       <c r="G26" s="30" t="inlineStr"/>
       <c r="H26" s="31">
@@ -8194,11 +8190,7 @@
           <t>Arbeit</t>
         </is>
       </c>
-      <c r="F27" s="30" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="F27" s="30" t="inlineStr"/>
       <c r="G27" s="30" t="inlineStr"/>
       <c r="H27" s="31">
         <f>IF($D27="ND",Настройки!$D$42,IF($D27="TD",Настройки!$D$39,""))</f>
@@ -8348,7 +8340,7 @@
       </c>
       <c r="D28" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>TD</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
@@ -8506,14 +8498,10 @@
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E29" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E29" s="30" t="inlineStr"/>
       <c r="F29" s="30" t="inlineStr"/>
       <c r="G29" s="30" t="inlineStr"/>
       <c r="H29" s="31">
@@ -8664,14 +8652,10 @@
       </c>
       <c r="D30" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E30" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E30" s="30" t="inlineStr"/>
       <c r="F30" s="30" t="inlineStr"/>
       <c r="G30" s="30" t="inlineStr"/>
       <c r="H30" s="31">
@@ -8822,10 +8806,14 @@
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E31" s="30" t="inlineStr"/>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="E31" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
       <c r="F31" s="30" t="inlineStr"/>
       <c r="G31" s="30" t="inlineStr"/>
       <c r="H31" s="31">
@@ -8984,11 +8972,7 @@
           <t>Arbeit</t>
         </is>
       </c>
-      <c r="F32" s="30" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="F32" s="30" t="inlineStr"/>
       <c r="G32" s="30" t="inlineStr"/>
       <c r="H32" s="31">
         <f>IF($D32="ND",Настройки!$D$42,IF($D32="TD",Настройки!$D$39,""))</f>
@@ -9138,14 +9122,10 @@
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E33" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E33" s="30" t="inlineStr"/>
       <c r="F33" s="30" t="inlineStr"/>
       <c r="G33" s="30" t="inlineStr"/>
       <c r="H33" s="31">
@@ -9296,14 +9276,10 @@
       </c>
       <c r="D34" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E34" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E34" s="30" t="inlineStr"/>
       <c r="F34" s="30" t="inlineStr"/>
       <c r="G34" s="30" t="inlineStr"/>
       <c r="H34" s="31">

</xml_diff>

<commit_message>
Record the employer's confirmed surcharge windows
The employer confirmed in writing that night runs 20:00-06:00, that
the Sunday surcharge starts at 00:00, and that a Sunday hour counts
as Sunday rather than night when the two overlap. That is what the
sheet already computes, so the notes now cite the confirmation
instead of leaving the windows looking like assumptions.

Also flags the one surcharge still unsettled: no payslip has yet
carried a public holiday, and the contract offers either +35 % with
time off in lieu or +135 % without. The first case falls on
03.10.2026, worth about 324 EUR gross either way.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NKeNmKEfCtXiZJGvjE51Zk
</commit_message>
<xml_diff>
--- a/Gehaltsrechner_Karimov.xlsx
+++ b/Gehaltsrechner_Karimov.xlsx
@@ -1609,7 +1609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2644,37 +2644,52 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="15" customHeight="1">
+    <row r="65" ht="39" customHeight="1">
       <c r="B65" s="5" t="inlineStr">
         <is>
+          <t>· Времена надбавок подтверждены работодателем письменно (Chris, WhatsApp, сентябрь 2026): ночь 20:00–06:00, воскресенье с 00:00, и при совпадении воскресенья с ночью считается ВОСКРЕСЕНЬЕ. Именно так файл и считает. Отсюда те 28 часов в августе, что ушли из ночных (25 %) в воскресные (50 %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="52" customHeight="1">
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>· ОТКРЫТО: как оплачивается ПРАЗДНИК. Договор § 3 Abs. 2 даёт +35 % с отгулом (c) или +135 % без отгула (d). Ни одной расчётки с праздником ещё не было. Первый случай — 03.10.2026, Tag der Deutschen Einheit: 12 праздничных часов, разница между вариантами ≈ 324 € брутто. Спросить заранее и проверить строку Feiertagszuschlag в расчётке за октябрь.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1">
+      <c r="B67" s="5" t="inlineStr">
+        <is>
           <t>· Доп. взнос кассы AOK Baden-Württemberg = 2,99 % (не средние 2,9 %). В «Настройках» исправлено.</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="15" customHeight="1">
-      <c r="B66" s="5" t="inlineStr">
+    <row r="68" ht="15" customHeight="1">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>· Доплата бездетным в Pflegeversicherung (0,6 %) не удерживается — ребёнок учтён правильно.</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="26" customHeight="1">
-      <c r="B67" s="5" t="inlineStr">
+    <row r="69" ht="26" customHeight="1">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>· Надбавки провели полностью свободными от взносов, хотя § 1 SvEV освобождает только с базы 25 €/ч. Сейчас это в твою пользу (~110 € в месяц), но уменьшает будущую пенсию на эту же базу.</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="26" customHeight="1">
-      <c r="B69" s="78" t="inlineStr">
+    <row r="71" ht="26" customHeight="1">
+      <c r="B71" s="78" t="inlineStr">
         <is>
           <t>Сроки, которые нельзя пропустить: по июлю — до 15.11.2026, по августу — до 14.12.2026. Разговор в WhatsApp сроки НЕ прерывает, нужна письменная претензия (e-mail достаточно).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="22">
     <mergeCell ref="B65:H65"/>
+    <mergeCell ref="B68:H68"/>
     <mergeCell ref="B64:H64"/>
     <mergeCell ref="B33:H33"/>
     <mergeCell ref="A1:H1"/>
@@ -2687,6 +2702,7 @@
     <mergeCell ref="B3:H3"/>
     <mergeCell ref="B66:H66"/>
     <mergeCell ref="B58:H58"/>
+    <mergeCell ref="B71:H71"/>
     <mergeCell ref="B21:H21"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B60:H60"/>
@@ -3073,7 +3089,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>20 = 20:00</t>
+          <t>20 = 20:00. Подтверждено работодателем (Chris, WhatsApp 09/2026): «20:00 – 06:00 morgens Nacht»</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3129,7 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>§ 3 Abs. 2 b)</t>
+          <t>§ 3 Abs. 2 b). Подтверждено (Chris): «Sonntags Zuschlag ab 00:00» и «Sonntag &gt; als Nacht, dann zählt Sonntag» — надбавки НЕ складываются</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update the September roster to the shifts actually worked
The month closed differently from the plan the sheet was built on:
27.09 and 28.09 lost their night shifts, and four day shifts were
added on 25, 28, 29 and 30. That makes 14 TD and 3 ND, 17 shifts of
12 h = 204 hours rather than 180, with 25.09 marked as eingesprungen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NKeNmKEfCtXiZJGvjE51Zk
</commit_message>
<xml_diff>
--- a/Gehaltsrechner_Karimov.xlsx
+++ b/Gehaltsrechner_Karimov.xlsx
@@ -816,7 +816,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>График месяца: ND / TD / FREI, статус (Arbeit / Urlaub / Krank), «x» = Eingesprungen. Сейчас заполнен СЕНТЯБРЬ 2026: 10 TD + 5 ND = 15 смен = 180 ч.</t>
+          <t>График месяца: ND / TD / FREI, статус (Arbeit / Urlaub / Krank), «x» = Eingesprungen. Сейчас заполнен СЕНТЯБРЬ 2026: 14 TD + 3 ND = 17 смен = 204 ч.</t>
         </is>
       </c>
     </row>
@@ -8514,11 +8514,19 @@
       </c>
       <c r="D29" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E29" s="30" t="inlineStr"/>
-      <c r="F29" s="30" t="inlineStr"/>
+          <t>TD</t>
+        </is>
+      </c>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
+      <c r="F29" s="30" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G29" s="30" t="inlineStr"/>
       <c r="H29" s="31">
         <f>IF($D29="ND",Настройки!$D$42,IF($D29="TD",Настройки!$D$39,""))</f>
@@ -8822,14 +8830,10 @@
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
-        </is>
-      </c>
-      <c r="E31" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E31" s="30" t="inlineStr"/>
       <c r="F31" s="30" t="inlineStr"/>
       <c r="G31" s="30" t="inlineStr"/>
       <c r="H31" s="31">
@@ -8980,7 +8984,7 @@
       </c>
       <c r="D32" s="30" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>TD</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
@@ -9138,10 +9142,14 @@
       </c>
       <c r="D33" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E33" s="30" t="inlineStr"/>
+          <t>TD</t>
+        </is>
+      </c>
+      <c r="E33" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
       <c r="F33" s="30" t="inlineStr"/>
       <c r="G33" s="30" t="inlineStr"/>
       <c r="H33" s="31">
@@ -9292,10 +9300,14 @@
       </c>
       <c r="D34" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E34" s="30" t="inlineStr"/>
+          <t>TD</t>
+        </is>
+      </c>
+      <c r="E34" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
       <c r="F34" s="30" t="inlineStr"/>
       <c r="G34" s="30" t="inlineStr"/>
       <c r="H34" s="31">

</xml_diff>

<commit_message>
Add the day shift picked up on 27.09
27.09 went from FREI to TD, making 18 shifts and 216 hours. It is a
Sunday, so the whole shift carries the 50 % surcharge and Sunday
hours rise from 24 to 36.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NKeNmKEfCtXiZJGvjE51Zk
</commit_message>
<xml_diff>
--- a/Gehaltsrechner_Karimov.xlsx
+++ b/Gehaltsrechner_Karimov.xlsx
@@ -816,7 +816,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>График месяца: ND / TD / FREI, статус (Arbeit / Urlaub / Krank), «x» = Eingesprungen. Сейчас заполнен СЕНТЯБРЬ 2026: 14 TD + 3 ND = 17 смен = 204 ч.</t>
+          <t>График месяца: ND / TD / FREI, статус (Arbeit / Urlaub / Krank), «x» = Eingesprungen. Сейчас заполнен СЕНТЯБРЬ 2026: 15 TD + 3 ND = 18 смен = 216 ч.</t>
         </is>
       </c>
     </row>
@@ -8830,10 +8830,14 @@
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>FREI</t>
-        </is>
-      </c>
-      <c r="E31" s="30" t="inlineStr"/>
+          <t>TD</t>
+        </is>
+      </c>
+      <c r="E31" s="30" t="inlineStr">
+        <is>
+          <t>Arbeit</t>
+        </is>
+      </c>
       <c r="F31" s="30" t="inlineStr"/>
       <c r="G31" s="30" t="inlineStr"/>
       <c r="H31" s="31">

</xml_diff>

<commit_message>
Drop the 27.09 shift that was never worked
It was entered in the roster app by mistake. Back to 17 shifts and
204 hours, which is what the September payslip settles, and the
Sunday hours match it at 24.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NKeNmKEfCtXiZJGvjE51Zk
</commit_message>
<xml_diff>
--- a/Gehaltsrechner_Karimov.xlsx
+++ b/Gehaltsrechner_Karimov.xlsx
@@ -816,7 +816,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>График месяца: ND / TD / FREI, статус (Arbeit / Urlaub / Krank), «x» = Eingesprungen. Сейчас заполнен СЕНТЯБРЬ 2026: 15 TD + 3 ND = 18 смен = 216 ч.</t>
+          <t>График месяца: ND / TD / FREI, статус (Arbeit / Urlaub / Krank), «x» = Eingesprungen. Сейчас заполнен СЕНТЯБРЬ 2026: 14 TD + 3 ND = 17 смен = 204 ч.</t>
         </is>
       </c>
     </row>
@@ -8830,14 +8830,10 @@
       </c>
       <c r="D31" s="30" t="inlineStr">
         <is>
-          <t>TD</t>
-        </is>
-      </c>
-      <c r="E31" s="30" t="inlineStr">
-        <is>
-          <t>Arbeit</t>
-        </is>
-      </c>
+          <t>FREI</t>
+        </is>
+      </c>
+      <c r="E31" s="30" t="inlineStr"/>
       <c r="F31" s="30" t="inlineStr"/>
       <c r="G31" s="30" t="inlineStr"/>
       <c r="H31" s="31">

</xml_diff>